<commit_message>
Update project with Codex
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -4,38 +4,57 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Sales Data" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Comparison" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Product</t>
-  </si>
-  <si>
-    <t>Price</t>
-  </si>
-  <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>Tea</t>
-  </si>
-  <si>
-    <t>Coffee</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="11">
+  <si>
+    <t>Валюта</t>
+  </si>
+  <si>
+    <t>Тип курсу</t>
+  </si>
+  <si>
+    <t>Курс (Minfin)</t>
+  </si>
+  <si>
+    <t>Курс (Kurs.com.ua)</t>
+  </si>
+  <si>
+    <t>Різниця (Minfin - Kurs)</t>
+  </si>
+  <si>
+    <t>Дата / Час</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>buy</t>
+  </si>
+  <si>
+    <t>2026-07-13T13:37:16.435Z</t>
+  </si>
+  <si>
+    <t>sell</t>
+  </si>
+  <si>
+    <t>EUR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0000;[Red]-0.0000"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -43,13 +62,22 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -64,8 +92,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -405,57 +436,119 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="4" width="15" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2">
+        <v>7</v>
+      </c>
+      <c r="C2" s="2">
+        <v>44.8</v>
+      </c>
+      <c r="D2" s="2">
+        <v>44.397</v>
+      </c>
+      <c r="E2" s="3">
+        <v>0.403</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2">
+        <v>44.83</v>
+      </c>
+      <c r="D3" s="2">
+        <v>44.864</v>
+      </c>
+      <c r="E3" s="3">
+        <v>-0.034</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>10</v>
       </c>
-      <c r="D2">
-        <v>2</v>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="2">
+        <v>51.2064</v>
+      </c>
+      <c r="D4" s="2">
+        <v>50.73</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0.4764</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3">
-        <v>15</v>
-      </c>
-      <c r="D3">
-        <v>3</v>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="2">
+        <v>51.2272</v>
+      </c>
+      <c r="D5" s="2">
+        <v>51.351</v>
+      </c>
+      <c r="E5" s="3">
+        <v>-0.1238</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>